<commit_message>
cloud sql vcpu and ram logic changed
</commit_message>
<xml_diff>
--- a/processed_data.xlsx
+++ b/processed_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR9"/>
+  <dimension ref="A1:AR11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -526,32 +526,32 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>SUD Price</t>
+          <t>Unnamed: 19</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>SUD URL</t>
+          <t>Unnamed: 20</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>One Year Price</t>
+          <t>Unnamed: 21</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>One Year URL</t>
+          <t>Unnamed: 22</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>three Year Price</t>
+          <t>Unnamed: 23</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>three Year URL</t>
+          <t>Unnamed: 24</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
@@ -652,15 +652,15 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>MySQL</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
         <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>PostgreSQL</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>4.24</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -674,10 +674,10 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H2" t="n">
-        <v>52</v>
+        <v>26</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -686,7 +686,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>asia-south1</t>
+          <t>asia-southeast1</t>
         </is>
       </c>
       <c r="K2" t="n">
@@ -701,10 +701,18 @@
         <v>5</v>
       </c>
       <c r="N2" t="n">
-        <v>730</v>
-      </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
+        <v>623</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>hours</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
@@ -732,15 +740,11 @@
       <c r="AO2" t="inlineStr"/>
       <c r="AP2" t="inlineStr"/>
       <c r="AQ2" t="inlineStr"/>
-      <c r="AR2" t="inlineStr">
-        <is>
-          <t>Storage amount cannot be less than 10.74</t>
-        </is>
-      </c>
+      <c r="AR2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -748,7 +752,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -762,23 +766,23 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="H3" t="n">
-        <v>104</v>
+        <v>52</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Non-HA</t>
+          <t>HA</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>asia-south1</t>
+          <t>us-east4</t>
         </is>
       </c>
       <c r="K3" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -789,18 +793,10 @@
         <v>5</v>
       </c>
       <c r="N3" t="n">
-        <v>623</v>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>hours</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>month</t>
-        </is>
-      </c>
+        <v>730</v>
+      </c>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
@@ -828,23 +824,19 @@
       <c r="AO3" t="inlineStr"/>
       <c r="AP3" t="inlineStr"/>
       <c r="AQ3" t="inlineStr"/>
-      <c r="AR3" t="inlineStr">
-        <is>
-          <t>Storage amount cannot be less than 10.74</t>
-        </is>
-      </c>
+      <c r="AR3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>MySQL</t>
+          <t>PostgreSQL</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2.04</v>
+        <v>1</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -858,10 +850,10 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="H4" t="n">
-        <v>208</v>
+        <v>104</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -870,11 +862,11 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>asia-south1</t>
+          <t>us-central1</t>
         </is>
       </c>
       <c r="K4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -885,10 +877,18 @@
         <v>5</v>
       </c>
       <c r="N4" t="n">
-        <v>730</v>
-      </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
+        <v>623</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>hours</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
@@ -920,7 +920,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1.02</v>
+        <v>2.04</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -938,14 +938,14 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>g1-small</t>
+          <t xml:space="preserve">custom </t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>208</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -954,7 +954,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>asia-south1</t>
+          <t>us-east4</t>
         </is>
       </c>
       <c r="K5" t="n">
@@ -1004,15 +1004,15 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>PostgreSQL</t>
+          <t>MySQL</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1.36</v>
+        <v>1.02</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1022,23 +1022,23 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">custom </t>
+          <t>g1-small</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Non-HA</t>
+          <t>HA</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>asia-south1</t>
+          <t>europe-west3</t>
         </is>
       </c>
       <c r="K6" t="n">
@@ -1084,15 +1084,11 @@
       <c r="AO6" t="inlineStr"/>
       <c r="AP6" t="inlineStr"/>
       <c r="AQ6" t="inlineStr"/>
-      <c r="AR6" t="inlineStr">
-        <is>
-          <t>Storage amount cannot be less than 10.74</t>
-        </is>
-      </c>
+      <c r="AR6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1110,49 +1106,39 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve">custom </t>
+          <t>f1-micro</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Non-HA</t>
+          <t>HA</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>asia-south1</t>
+          <t>europe-west3</t>
         </is>
       </c>
       <c r="K7" t="n">
-        <v>10</v>
+        <v>256</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
           <t>HDD</t>
         </is>
       </c>
-      <c r="M7" t="n">
-        <v>5</v>
-      </c>
+      <c r="M7" t="inlineStr"/>
       <c r="N7" t="n">
-        <v>492</v>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>hours</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>month</t>
-        </is>
-      </c>
+        <v>730</v>
+      </c>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
@@ -1184,7 +1170,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -1192,7 +1178,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>4.08</v>
+        <v>1.36</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1222,7 +1208,7 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -1264,23 +1250,19 @@
       <c r="AO8" t="inlineStr"/>
       <c r="AP8" t="inlineStr"/>
       <c r="AQ8" t="inlineStr"/>
-      <c r="AR8" t="inlineStr">
-        <is>
-          <t>Storage amount cannot be less than 10.74</t>
-        </is>
-      </c>
+      <c r="AR8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PostgreSQL</t>
+          <t>MySQL</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>5.1</v>
+        <v>1</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1306,7 +1288,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>asia-south1</t>
+          <t>europe-west3</t>
         </is>
       </c>
       <c r="K9" t="n">
@@ -1321,10 +1303,18 @@
         <v>5</v>
       </c>
       <c r="N9" t="n">
-        <v>730</v>
-      </c>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
+        <v>492</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>hours</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr"/>
@@ -1352,11 +1342,175 @@
       <c r="AO9" t="inlineStr"/>
       <c r="AP9" t="inlineStr"/>
       <c r="AQ9" t="inlineStr"/>
-      <c r="AR9" t="inlineStr">
-        <is>
-          <t>Storage amount cannot be less than 10.74</t>
-        </is>
-      </c>
+      <c r="AR9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>14</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>PostgreSQL</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Enterprise</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">custom </t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" t="n">
+        <v>13</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>HA</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>asia-south1</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>11</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>HDD</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>5</v>
+      </c>
+      <c r="N10" t="n">
+        <v>730</v>
+      </c>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
+      <c r="X10" t="inlineStr"/>
+      <c r="Y10" t="inlineStr"/>
+      <c r="Z10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr"/>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr"/>
+      <c r="AD10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr"/>
+      <c r="AG10" t="inlineStr"/>
+      <c r="AH10" t="inlineStr"/>
+      <c r="AI10" t="inlineStr"/>
+      <c r="AJ10" t="inlineStr"/>
+      <c r="AK10" t="inlineStr"/>
+      <c r="AL10" t="inlineStr"/>
+      <c r="AM10" t="inlineStr"/>
+      <c r="AN10" t="inlineStr"/>
+      <c r="AO10" t="inlineStr"/>
+      <c r="AP10" t="inlineStr"/>
+      <c r="AQ10" t="inlineStr"/>
+      <c r="AR10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>15</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>PostgreSQL</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Enterprise</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">custom </t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>4</v>
+      </c>
+      <c r="H11" t="n">
+        <v>26</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Non-HA</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>us-east4</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>11</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>HDD</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>5</v>
+      </c>
+      <c r="N11" t="n">
+        <v>730</v>
+      </c>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr"/>
+      <c r="X11" t="inlineStr"/>
+      <c r="Y11" t="inlineStr"/>
+      <c r="Z11" t="inlineStr"/>
+      <c r="AA11" t="inlineStr"/>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr"/>
+      <c r="AD11" t="inlineStr"/>
+      <c r="AE11" t="inlineStr"/>
+      <c r="AF11" t="inlineStr"/>
+      <c r="AG11" t="inlineStr"/>
+      <c r="AH11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr"/>
+      <c r="AJ11" t="inlineStr"/>
+      <c r="AK11" t="inlineStr"/>
+      <c r="AL11" t="inlineStr"/>
+      <c r="AM11" t="inlineStr"/>
+      <c r="AN11" t="inlineStr"/>
+      <c r="AO11" t="inlineStr"/>
+      <c r="AP11" t="inlineStr"/>
+      <c r="AQ11" t="inlineStr"/>
+      <c r="AR11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>